<commit_message>
Fixed the sequence number
</commit_message>
<xml_diff>
--- a/product family/CMX/CMX 32 CKT (34868)/BOM.xlsx
+++ b/product family/CMX/CMX 32 CKT (34868)/BOM.xlsx
@@ -603,10 +603,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H4" t="n">
         <v>348681001</v>
@@ -639,10 +639,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H5" t="n">
         <v>348681001</v>
@@ -675,10 +675,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H6" t="n">
         <v>348681001</v>
@@ -711,10 +711,10 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H7" t="n">
         <v>348681001</v>
@@ -783,10 +783,10 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9" t="n">
         <v>348681002</v>
@@ -819,10 +819,10 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H10" t="n">
         <v>348681002</v>
@@ -855,10 +855,10 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H11" t="n">
         <v>348681002</v>
@@ -891,10 +891,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G12" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H12" t="n">
         <v>348681002</v>
@@ -927,10 +927,10 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G13" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H13" t="n">
         <v>348681002</v>
@@ -999,10 +999,10 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H15" t="n">
         <v>348681003</v>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H16" t="n">
         <v>348681003</v>
@@ -1071,10 +1071,10 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H17" t="n">
         <v>348681003</v>
@@ -1107,10 +1107,10 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G18" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H18" t="n">
         <v>348681003</v>
@@ -1143,10 +1143,10 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G19" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H19" t="n">
         <v>348681003</v>
@@ -1251,10 +1251,10 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H22" t="n">
         <v>348682001</v>
@@ -1287,10 +1287,10 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H23" t="n">
         <v>348682001</v>
@@ -1323,10 +1323,10 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H24" t="n">
         <v>348682001</v>
@@ -1359,10 +1359,10 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H25" t="n">
         <v>348682001</v>
@@ -1431,10 +1431,10 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H27" t="n">
         <v>348682002</v>
@@ -1467,10 +1467,10 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G28" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H28" t="n">
         <v>348682002</v>
@@ -1503,10 +1503,10 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G29" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H29" t="n">
         <v>348682002</v>
@@ -1539,10 +1539,10 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G30" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H30" t="n">
         <v>348682002</v>
@@ -1575,10 +1575,10 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G31" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H31" t="n">
         <v>348682002</v>
@@ -1647,10 +1647,10 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H33" t="n">
         <v>348682003</v>
@@ -1683,10 +1683,10 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H34" t="n">
         <v>348682003</v>
@@ -1719,10 +1719,10 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G35" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H35" t="n">
         <v>348682003</v>
@@ -1755,10 +1755,10 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G36" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H36" t="n">
         <v>348682003</v>
@@ -1791,10 +1791,10 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G37" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H37" t="n">
         <v>348682003</v>

</xml_diff>